<commit_message>
Backup QR Scanner data - 2026-03-03T08:25:56.174Z - Cache Bust: 1772526356174
</commit_message>
<xml_diff>
--- a/log_history/Y1_B2526_Pharmacology_scanner1772523701414_4791e799a156631a1e6528d73ff0b32fbeeb62851b63d680bacede618e9287f5.xlsx
+++ b/log_history/Y1_B2526_Pharmacology_scanner1772523701414_4791e799a156631a1e6528d73ff0b32fbeeb62851b63d680bacede618e9287f5.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Pharmacology" sheetId="1" r:id="rId1"/>
+    <sheet name="Scanner" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F51"/>
+  <dimension ref="A1:F53"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1419,9 +1419,49 @@
         <v>marian.samir@med.asu.edu.eg</v>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>254762</v>
+      </c>
+      <c r="B52" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C52" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D52" t="str">
+        <v>10:21:16</v>
+      </c>
+      <c r="E52" t="str">
+        <v>Manual</v>
+      </c>
+      <c r="F52" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>254716</v>
+      </c>
+      <c r="B53" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C53" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D53" t="str">
+        <v>10:21:21</v>
+      </c>
+      <c r="E53" t="str">
+        <v>Manual</v>
+      </c>
+      <c r="F53" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F51"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F53"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>